<commit_message>
working on the new irrigation log importing
--
</commit_message>
<xml_diff>
--- a/Penman_irrigation_results.xlsx
+++ b/Penman_irrigation_results.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC53"/>
+  <dimension ref="A1:BC54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9378,6 +9378,105 @@
         <v>19.4368</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH54" t="n">
+        <v>24</v>
+      </c>
+      <c r="AI54" t="n">
+        <v>24</v>
+      </c>
+      <c r="AJ54" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="AK54" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="AL54" t="inlineStr"/>
+      <c r="AM54" t="inlineStr"/>
+      <c r="AN54" t="inlineStr"/>
+      <c r="AO54" t="inlineStr"/>
+      <c r="AP54" t="inlineStr"/>
+      <c r="AQ54" t="inlineStr"/>
+      <c r="AR54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX54" t="inlineStr"/>
+      <c r="AY54" t="inlineStr"/>
+      <c r="AZ54" t="inlineStr"/>
+      <c r="BA54" t="inlineStr"/>
+      <c r="BB54" t="inlineStr"/>
+      <c r="BC54" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>